<commit_message>
Tambahkan workspace operator UP/TUP dan KKP
- Arahkan menu ke `/operator/up-tup` dengan skor aktual, dampak rencana,
  reminder GUP/PTUP, dan panel simulasi GUP/KKP
- Tambahkan helper workspace serta test mapping actual, skor, merge asumsi,
  dan reminder jatuh tempo
- Lengkapi panel asumsi dengan preview kualitas GUP, tabel acuan, dan catatan
  operasional dari referensi Excel
</commit_message>
<xml_diff>
--- a/referensi/Referensi UP GUP KKP.xlsx
+++ b/referensi/Referensi UP GUP KKP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Vibe Coding\simulator-ikpa\referensi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930B916C-0EFF-439B-9669-DD10C20E472E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B5B085-B35A-4E66-908C-F418B42F618F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simulasi Setiap GUP" sheetId="5" r:id="rId1"/>
@@ -225,10 +225,10 @@
   <numFmts count="6">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;hari&quot;"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0\ &quot;hari&quot;"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -631,13 +631,13 @@
     <xf numFmtId="9" fontId="10" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="5" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -650,15 +650,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="6" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="11" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -723,6 +723,43 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -752,43 +789,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1152,7 +1152,7 @@
     <col min="4" max="4" width="21.5703125" style="3" customWidth="1"/>
     <col min="5" max="5" width="33.140625" style="3" customWidth="1"/>
     <col min="6" max="6" width="7.140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="20" style="3" customWidth="1"/>
     <col min="8" max="10" width="14.140625" style="3" customWidth="1"/>
     <col min="11" max="13" width="11.85546875" style="3" customWidth="1"/>
     <col min="14" max="14" width="8.7109375" style="3" customWidth="1"/>
@@ -1212,22 +1212,22 @@
     </row>
     <row r="4" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="61"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="76"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="62" t="s">
+      <c r="G4" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
-      <c r="L4" s="63"/>
-      <c r="M4" s="63"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
+      <c r="L4" s="78"/>
+      <c r="M4" s="78"/>
       <c r="N4" s="4"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
@@ -1244,24 +1244,24 @@
     </row>
     <row r="5" spans="1:26" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="58"/>
-      <c r="D5" s="58"/>
-      <c r="E5" s="56"/>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="71"/>
       <c r="F5" s="4"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="65" t="s">
+      <c r="H5" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="66"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="68" t="s">
+      <c r="I5" s="81"/>
+      <c r="J5" s="82"/>
+      <c r="K5" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="L5" s="66"/>
-      <c r="M5" s="67"/>
+      <c r="L5" s="81"/>
+      <c r="M5" s="82"/>
       <c r="N5" s="4"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
@@ -1278,12 +1278,12 @@
     </row>
     <row r="6" spans="1:26" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
-      <c r="B6" s="69" t="s">
+      <c r="B6" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="56"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="71"/>
       <c r="F6" s="4"/>
       <c r="G6" s="7" t="s">
         <v>7</v>
@@ -1450,7 +1450,7 @@
         <v>10</v>
       </c>
       <c r="C10" s="26">
-        <v>18000000</v>
+        <v>1000000</v>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="24"/>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="C11" s="27">
         <f>C10/C9</f>
-        <v>1</v>
+        <v>5.5555555555555552E-2</v>
       </c>
       <c r="D11" s="23"/>
       <c r="E11" s="24"/>
@@ -1893,13 +1893,13 @@
       </c>
       <c r="C19" s="39">
         <f>C11*(E14/E17)</f>
-        <v>1.55</v>
-      </c>
-      <c r="D19" s="55" t="str">
+        <v>8.611111111111111E-2</v>
+      </c>
+      <c r="D19" s="70" t="str">
         <f>IF(C19&lt;100%,"UBAH Tanggal Rencana GUP (SP2D) LEBIH CEPAT ATAU Nilai Rencana GUP DITAMBAHKAN","OKE")</f>
-        <v>OKE</v>
-      </c>
-      <c r="E19" s="56"/>
+        <v>UBAH Tanggal Rencana GUP (SP2D) LEBIH CEPAT ATAU Nilai Rencana GUP DITAMBAHKAN</v>
+      </c>
+      <c r="E19" s="71"/>
       <c r="F19" s="4"/>
       <c r="G19" s="40"/>
       <c r="H19" s="40"/>
@@ -1927,7 +1927,7 @@
       <c r="B20" s="42"/>
       <c r="C20" s="43" t="str">
         <f>IF(C19&gt;=100%,"MAKSIMAL NILAI ADALAH 100%","-")</f>
-        <v>MAKSIMAL NILAI ADALAH 100%</v>
+        <v>-</v>
       </c>
       <c r="D20" s="44"/>
       <c r="E20" s="45"/>
@@ -2103,12 +2103,12 @@
     </row>
     <row r="26" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="51"/>
-      <c r="B26" s="57" t="s">
+      <c r="B26" s="72" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="58"/>
-      <c r="D26" s="58"/>
-      <c r="E26" s="58"/>
+      <c r="C26" s="73"/>
+      <c r="D26" s="73"/>
+      <c r="E26" s="73"/>
       <c r="F26" s="52"/>
       <c r="G26" s="52"/>
       <c r="H26" s="53"/>
@@ -8551,15 +8551,15 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16" style="70" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="70" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="71"/>
-    <col min="5" max="5" width="14.85546875" style="72" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="73" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" style="73" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" style="73" customWidth="1"/>
+    <col min="2" max="2" width="16" style="55" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" style="55" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="56"/>
+    <col min="5" max="5" width="14.85546875" style="57" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" style="58" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" style="58" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" style="58" customWidth="1"/>
     <col min="10" max="10" width="10.7109375" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="74"/>
+    <col min="11" max="11" width="9.140625" style="59"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -8568,68 +8568,68 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="76" t="s">
+      <c r="C3" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="75" t="s">
+      <c r="D3" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="75"/>
-      <c r="F3" s="76" t="s">
+      <c r="E3" s="69"/>
+      <c r="F3" s="68" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="76" t="s">
+      <c r="G3" s="68" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="76" t="s">
+      <c r="H3" s="68" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="77" t="s">
+      <c r="A4" s="69"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="77" t="s">
+      <c r="E4" s="60" t="s">
         <v>33</v>
       </c>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
+      <c r="F4" s="68"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="68"/>
     </row>
     <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="78">
+      <c r="A5" s="61">
         <v>1</v>
       </c>
-      <c r="B5" s="79">
+      <c r="B5" s="62">
         <v>0</v>
       </c>
-      <c r="C5" s="79">
+      <c r="C5" s="62">
         <f>B5*12</f>
         <v>0</v>
       </c>
-      <c r="D5" s="80">
+      <c r="D5" s="63">
         <v>0.01</v>
       </c>
-      <c r="E5" s="81">
+      <c r="E5" s="64">
         <f>D5*C5</f>
         <v>0</v>
       </c>
-      <c r="F5" s="82">
+      <c r="F5" s="65">
         <v>0</v>
       </c>
-      <c r="G5" s="82">
+      <c r="G5" s="65">
         <v>0</v>
       </c>
-      <c r="H5" s="82">
+      <c r="H5" s="65">
         <v>0</v>
       </c>
       <c r="J5" t="s">
@@ -8637,26 +8637,26 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="78">
+      <c r="A6" s="61">
         <v>2</v>
       </c>
-      <c r="B6" s="79">
+      <c r="B6" s="62">
         <v>0</v>
       </c>
-      <c r="C6" s="79">
+      <c r="C6" s="62">
         <f t="shared" ref="C6:C16" si="0">B6*12</f>
         <v>0</v>
       </c>
-      <c r="D6" s="80">
+      <c r="D6" s="63">
         <v>0.01</v>
       </c>
-      <c r="E6" s="81">
+      <c r="E6" s="64">
         <f t="shared" ref="E6:E16" si="1">D6*C6</f>
         <v>0</v>
       </c>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="82">
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65">
         <v>0</v>
       </c>
       <c r="J6" t="s">
@@ -8664,247 +8664,247 @@
       </c>
     </row>
     <row r="7" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="78">
+      <c r="A7" s="61">
         <v>3</v>
       </c>
-      <c r="B7" s="79">
+      <c r="B7" s="62">
         <v>0</v>
       </c>
-      <c r="C7" s="79">
+      <c r="C7" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D7" s="80">
+      <c r="D7" s="63">
         <v>0.01</v>
       </c>
-      <c r="E7" s="81">
+      <c r="E7" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F7" s="82"/>
-      <c r="G7" s="82"/>
-      <c r="H7" s="82">
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65">
         <v>0</v>
       </c>
       <c r="J7" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="74">
+      <c r="K7" s="59">
         <v>99.06</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="78">
+      <c r="A8" s="61">
         <v>4</v>
       </c>
-      <c r="B8" s="79">
+      <c r="B8" s="62">
         <v>0</v>
       </c>
-      <c r="C8" s="79">
+      <c r="C8" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D8" s="80">
+      <c r="D8" s="63">
         <v>0.05</v>
       </c>
-      <c r="E8" s="81">
+      <c r="E8" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
-      <c r="H8" s="82"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="65"/>
       <c r="J8" t="s">
         <v>37</v>
       </c>
-      <c r="K8" s="74">
+      <c r="K8" s="59">
         <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="78">
+      <c r="A9" s="61">
         <v>5</v>
       </c>
-      <c r="B9" s="79">
+      <c r="B9" s="62">
         <v>0</v>
       </c>
-      <c r="C9" s="79">
+      <c r="C9" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D9" s="80">
+      <c r="D9" s="63">
         <v>0.05</v>
       </c>
-      <c r="E9" s="81">
+      <c r="E9" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
-      <c r="H9" s="82"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
       <c r="J9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="78">
+      <c r="A10" s="61">
         <v>6</v>
       </c>
-      <c r="B10" s="79">
+      <c r="B10" s="62">
         <v>0</v>
       </c>
-      <c r="C10" s="79">
+      <c r="C10" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D10" s="80">
+      <c r="D10" s="63">
         <v>0.05</v>
       </c>
-      <c r="E10" s="81">
+      <c r="E10" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F10" s="82"/>
-      <c r="G10" s="82"/>
-      <c r="H10" s="82">
+      <c r="F10" s="65"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="65">
         <v>110</v>
       </c>
-      <c r="J10" s="83">
+      <c r="J10" s="66">
         <f>(K7*90%)+(K8*10%)</f>
         <v>100.15400000000001</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="78">
+      <c r="A11" s="61">
         <v>7</v>
       </c>
-      <c r="B11" s="79">
+      <c r="B11" s="62">
         <v>0</v>
       </c>
-      <c r="C11" s="79">
+      <c r="C11" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D11" s="80">
+      <c r="D11" s="63">
         <v>0.09</v>
       </c>
-      <c r="E11" s="81">
+      <c r="E11" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-      <c r="H11" s="82"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
     </row>
     <row r="12" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="78">
+      <c r="A12" s="61">
         <v>8</v>
       </c>
-      <c r="B12" s="79">
+      <c r="B12" s="62">
         <v>0</v>
       </c>
-      <c r="C12" s="79">
+      <c r="C12" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D12" s="80">
+      <c r="D12" s="63">
         <v>0.09</v>
       </c>
-      <c r="E12" s="81">
+      <c r="E12" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F12" s="82"/>
-      <c r="G12" s="82"/>
-      <c r="H12" s="82"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
     </row>
     <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="78">
+      <c r="A13" s="61">
         <v>9</v>
       </c>
-      <c r="B13" s="79">
+      <c r="B13" s="62">
         <v>0</v>
       </c>
-      <c r="C13" s="79">
+      <c r="C13" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D13" s="80">
+      <c r="D13" s="63">
         <v>0.09</v>
       </c>
-      <c r="E13" s="81">
+      <c r="E13" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F13" s="82"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="82"/>
+      <c r="F13" s="65"/>
+      <c r="G13" s="65"/>
+      <c r="H13" s="65"/>
     </row>
     <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="78">
+      <c r="A14" s="61">
         <v>10</v>
       </c>
-      <c r="B14" s="79">
+      <c r="B14" s="62">
         <v>0</v>
       </c>
-      <c r="C14" s="79">
+      <c r="C14" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D14" s="84">
+      <c r="D14" s="67">
         <v>0.125</v>
       </c>
-      <c r="E14" s="81">
+      <c r="E14" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F14" s="82"/>
-      <c r="G14" s="82"/>
-      <c r="H14" s="82"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
     </row>
     <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="78">
+      <c r="A15" s="61">
         <v>11</v>
       </c>
-      <c r="B15" s="79">
+      <c r="B15" s="62">
         <v>0</v>
       </c>
-      <c r="C15" s="79">
+      <c r="C15" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D15" s="84">
+      <c r="D15" s="67">
         <v>0.125</v>
       </c>
-      <c r="E15" s="81">
+      <c r="E15" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F15" s="82"/>
-      <c r="G15" s="82"/>
-      <c r="H15" s="82"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="65"/>
     </row>
     <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="78">
+      <c r="A16" s="61">
         <v>12</v>
       </c>
-      <c r="B16" s="79">
+      <c r="B16" s="62">
         <v>0</v>
       </c>
-      <c r="C16" s="79">
+      <c r="C16" s="62">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D16" s="84">
+      <c r="D16" s="67">
         <v>0.125</v>
       </c>
-      <c r="E16" s="81">
+      <c r="E16" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-      <c r="H16" s="82"/>
+      <c r="F16" s="65"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -8921,17 +8921,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="0ef7128f-a7d0-43d2-bee4-5f56f49c64da" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6d95bc28-2e5c-4ccd-92aa-ea746d833732">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003A8A126F045CFA4FBFC051756F52F0CC" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3208e68b71c22743ea86da60d1e9ab54">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6d95bc28-2e5c-4ccd-92aa-ea746d833732" xmlns:ns3="0ef7128f-a7d0-43d2-bee4-5f56f49c64da" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2fefb0d127e3815082eddebadb8446cd" ns2:_="" ns3:_="">
     <xsd:import namespace="6d95bc28-2e5c-4ccd-92aa-ea746d833732"/>
@@ -9166,6 +9155,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="0ef7128f-a7d0-43d2-bee4-5f56f49c64da" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6d95bc28-2e5c-4ccd-92aa-ea746d833732">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9176,17 +9176,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66C24C32-26A5-46B6-8905-74C1706A1B8E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0ef7128f-a7d0-43d2-bee4-5f56f49c64da"/>
-    <ds:schemaRef ds:uri="6d95bc28-2e5c-4ccd-92aa-ea746d833732"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1525FCB5-2927-4CB5-A0D1-7D9C8097191F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9205,6 +9194,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66C24C32-26A5-46B6-8905-74C1706A1B8E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0ef7128f-a7d0-43d2-bee4-5f56f49c64da"/>
+    <ds:schemaRef ds:uri="6d95bc28-2e5c-4ccd-92aa-ea746d833732"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BB4633B-1A3C-4046-B120-75C7A0D242D0}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat: sederhanakan form UP/TUP dan konsolidasikan tab KKP
</commit_message>
<xml_diff>
--- a/referensi/Referensi UP GUP KKP.xlsx
+++ b/referensi/Referensi UP GUP KKP.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Vibe Coding\simulator-ikpa\referensi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B5B085-B35A-4E66-908C-F418B42F618F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2CD947-EACB-492B-9B80-DEF627B3C96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Simulasi Setiap GUP" sheetId="5" r:id="rId1"/>
-    <sheet name="UP KKP" sheetId="6" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>SILAHKAN KLIK FILE - BUAT SALINAN/MAKE A COPY ATAU KLIK FILE - DOWNLOAD</t>
   </si>
@@ -172,73 +171,17 @@
   <si>
     <t>Copyright Subbagian Perbendaharaan - Bagian Keuangan - Sekretariat DJPb</t>
   </si>
-  <si>
-    <t>Perhitungan UP KKP Satker</t>
-  </si>
-  <si>
-    <t>Periode</t>
-  </si>
-  <si>
-    <t>UP KKP/bulan</t>
-  </si>
-  <si>
-    <t>UP KKP 1 tahun</t>
-  </si>
-  <si>
-    <t>Target Penggunaan KKP</t>
-  </si>
-  <si>
-    <t>Penggunaan KKP (kumulatif)</t>
-  </si>
-  <si>
-    <t>Nilai Kinerja Penggunaan KKP</t>
-  </si>
-  <si>
-    <t>Nilai Komponen UP KKP</t>
-  </si>
-  <si>
-    <t>% Target</t>
-  </si>
-  <si>
-    <t>Nominal Target</t>
-  </si>
-  <si>
-    <t>Nilai IKPA :</t>
-  </si>
-  <si>
-    <t>(NK Tunai x 90%) + (NK KKP x 10%)</t>
-  </si>
-  <si>
-    <t>NK Tunai  :</t>
-  </si>
-  <si>
-    <t>NK KKP :</t>
-  </si>
-  <si>
-    <t>IKPA :</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0\ &quot;hari&quot;"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -345,13 +288,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -433,7 +369,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -582,218 +518,164 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="9" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="7" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="10" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="5" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="14" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{17E562A6-D755-43EA-B313-2C37AB88CB2B}"/>
   </cellStyles>
@@ -1212,22 +1094,22 @@
     </row>
     <row r="4" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="B4" s="74" t="s">
+      <c r="B4" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="76"/>
+      <c r="C4" s="60"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="61"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="77" t="s">
+      <c r="G4" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="78"/>
-      <c r="I4" s="78"/>
-      <c r="J4" s="78"/>
-      <c r="K4" s="78"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="78"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63"/>
+      <c r="M4" s="63"/>
       <c r="N4" s="4"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
@@ -1244,24 +1126,24 @@
     </row>
     <row r="5" spans="1:26" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
-      <c r="B5" s="79" t="s">
+      <c r="B5" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="73"/>
-      <c r="D5" s="73"/>
-      <c r="E5" s="71"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="56"/>
       <c r="F5" s="4"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="80" t="s">
+      <c r="H5" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="81"/>
-      <c r="J5" s="82"/>
-      <c r="K5" s="83" t="s">
+      <c r="I5" s="66"/>
+      <c r="J5" s="67"/>
+      <c r="K5" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="L5" s="81"/>
-      <c r="M5" s="82"/>
+      <c r="L5" s="66"/>
+      <c r="M5" s="67"/>
       <c r="N5" s="4"/>
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
@@ -1278,12 +1160,12 @@
     </row>
     <row r="6" spans="1:26" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="73"/>
-      <c r="D6" s="73"/>
-      <c r="E6" s="71"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="56"/>
       <c r="F6" s="4"/>
       <c r="G6" s="7" t="s">
         <v>7</v>
@@ -1895,11 +1777,11 @@
         <f>C11*(E14/E17)</f>
         <v>8.611111111111111E-2</v>
       </c>
-      <c r="D19" s="70" t="str">
+      <c r="D19" s="55" t="str">
         <f>IF(C19&lt;100%,"UBAH Tanggal Rencana GUP (SP2D) LEBIH CEPAT ATAU Nilai Rencana GUP DITAMBAHKAN","OKE")</f>
         <v>UBAH Tanggal Rencana GUP (SP2D) LEBIH CEPAT ATAU Nilai Rencana GUP DITAMBAHKAN</v>
       </c>
-      <c r="E19" s="71"/>
+      <c r="E19" s="56"/>
       <c r="F19" s="4"/>
       <c r="G19" s="40"/>
       <c r="H19" s="40"/>
@@ -2103,12 +1985,12 @@
     </row>
     <row r="26" spans="1:26" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="51"/>
-      <c r="B26" s="72" t="s">
+      <c r="B26" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="73"/>
-      <c r="D26" s="73"/>
-      <c r="E26" s="73"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
       <c r="F26" s="52"/>
       <c r="G26" s="52"/>
       <c r="H26" s="53"/>
@@ -8545,382 +8427,27 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1311DD04-3505-409C-9FC8-D985F19E416A}">
-  <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16" style="55" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="55" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="56"/>
-    <col min="5" max="5" width="14.85546875" style="57" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="58" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" style="58" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" style="58" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="59"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="69" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="68" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="68" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="69" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="69"/>
-      <c r="F3" s="68" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="68" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" s="68" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="69"/>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="60" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-    </row>
-    <row r="5" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="61">
-        <v>1</v>
-      </c>
-      <c r="B5" s="62">
-        <v>0</v>
-      </c>
-      <c r="C5" s="62">
-        <f>B5*12</f>
-        <v>0</v>
-      </c>
-      <c r="D5" s="63">
-        <v>0.01</v>
-      </c>
-      <c r="E5" s="64">
-        <f>D5*C5</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="65">
-        <v>0</v>
-      </c>
-      <c r="G5" s="65">
-        <v>0</v>
-      </c>
-      <c r="H5" s="65">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="61">
-        <v>2</v>
-      </c>
-      <c r="B6" s="62">
-        <v>0</v>
-      </c>
-      <c r="C6" s="62">
-        <f t="shared" ref="C6:C16" si="0">B6*12</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="63">
-        <v>0.01</v>
-      </c>
-      <c r="E6" s="64">
-        <f t="shared" ref="E6:E16" si="1">D6*C6</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65">
-        <v>0</v>
-      </c>
-      <c r="J6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="61">
-        <v>3</v>
-      </c>
-      <c r="B7" s="62">
-        <v>0</v>
-      </c>
-      <c r="C7" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D7" s="63">
-        <v>0.01</v>
-      </c>
-      <c r="E7" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="65">
-        <v>0</v>
-      </c>
-      <c r="J7" t="s">
-        <v>36</v>
-      </c>
-      <c r="K7" s="59">
-        <v>99.06</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="61">
-        <v>4</v>
-      </c>
-      <c r="B8" s="62">
-        <v>0</v>
-      </c>
-      <c r="C8" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D8" s="63">
-        <v>0.05</v>
-      </c>
-      <c r="E8" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="65"/>
-      <c r="G8" s="65"/>
-      <c r="H8" s="65"/>
-      <c r="J8" t="s">
-        <v>37</v>
-      </c>
-      <c r="K8" s="59">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="61">
-        <v>5</v>
-      </c>
-      <c r="B9" s="62">
-        <v>0</v>
-      </c>
-      <c r="C9" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D9" s="63">
-        <v>0.05</v>
-      </c>
-      <c r="E9" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
-      <c r="J9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="61">
-        <v>6</v>
-      </c>
-      <c r="B10" s="62">
-        <v>0</v>
-      </c>
-      <c r="C10" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D10" s="63">
-        <v>0.05</v>
-      </c>
-      <c r="E10" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="65"/>
-      <c r="G10" s="65"/>
-      <c r="H10" s="65">
-        <v>110</v>
-      </c>
-      <c r="J10" s="66">
-        <f>(K7*90%)+(K8*10%)</f>
-        <v>100.15400000000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="61">
-        <v>7</v>
-      </c>
-      <c r="B11" s="62">
-        <v>0</v>
-      </c>
-      <c r="C11" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D11" s="63">
-        <v>0.09</v>
-      </c>
-      <c r="E11" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
-    </row>
-    <row r="12" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="61">
-        <v>8</v>
-      </c>
-      <c r="B12" s="62">
-        <v>0</v>
-      </c>
-      <c r="C12" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D12" s="63">
-        <v>0.09</v>
-      </c>
-      <c r="E12" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-    </row>
-    <row r="13" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="61">
-        <v>9</v>
-      </c>
-      <c r="B13" s="62">
-        <v>0</v>
-      </c>
-      <c r="C13" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D13" s="63">
-        <v>0.09</v>
-      </c>
-      <c r="E13" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F13" s="65"/>
-      <c r="G13" s="65"/>
-      <c r="H13" s="65"/>
-    </row>
-    <row r="14" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="61">
-        <v>10</v>
-      </c>
-      <c r="B14" s="62">
-        <v>0</v>
-      </c>
-      <c r="C14" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D14" s="67">
-        <v>0.125</v>
-      </c>
-      <c r="E14" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F14" s="65"/>
-      <c r="G14" s="65"/>
-      <c r="H14" s="65"/>
-    </row>
-    <row r="15" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="61">
-        <v>11</v>
-      </c>
-      <c r="B15" s="62">
-        <v>0</v>
-      </c>
-      <c r="C15" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D15" s="67">
-        <v>0.125</v>
-      </c>
-      <c r="E15" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="65"/>
-    </row>
-    <row r="16" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="61">
-        <v>12</v>
-      </c>
-      <c r="B16" s="62">
-        <v>0</v>
-      </c>
-      <c r="C16" s="62">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="D16" s="67">
-        <v>0.125</v>
-      </c>
-      <c r="E16" s="64">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F16" s="65"/>
-      <c r="G16" s="65"/>
-      <c r="H16" s="65"/>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="0ef7128f-a7d0-43d2-bee4-5f56f49c64da" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6d95bc28-2e5c-4ccd-92aa-ea746d833732">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003A8A126F045CFA4FBFC051756F52F0CC" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3208e68b71c22743ea86da60d1e9ab54">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6d95bc28-2e5c-4ccd-92aa-ea746d833732" xmlns:ns3="0ef7128f-a7d0-43d2-bee4-5f56f49c64da" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2fefb0d127e3815082eddebadb8446cd" ns2:_="" ns3:_="">
     <xsd:import namespace="6d95bc28-2e5c-4ccd-92aa-ea746d833732"/>
@@ -9155,27 +8682,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="0ef7128f-a7d0-43d2-bee4-5f56f49c64da" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6d95bc28-2e5c-4ccd-92aa-ea746d833732">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BB4633B-1A3C-4046-B120-75C7A0D242D0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66C24C32-26A5-46B6-8905-74C1706A1B8E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0ef7128f-a7d0-43d2-bee4-5f56f49c64da"/>
+    <ds:schemaRef ds:uri="6d95bc28-2e5c-4ccd-92aa-ea746d833732"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1525FCB5-2927-4CB5-A0D1-7D9C8097191F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9194,25 +8720,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66C24C32-26A5-46B6-8905-74C1706A1B8E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0ef7128f-a7d0-43d2-bee4-5f56f49c64da"/>
-    <ds:schemaRef ds:uri="6d95bc28-2e5c-4ccd-92aa-ea746d833732"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BB4633B-1A3C-4046-B120-75C7A0D242D0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{ed6fb366-8322-46f3-915e-c4d037a454a9}" enabled="0" method="" siteId="{ed6fb366-8322-46f3-915e-c4d037a454a9}" removed="1"/>

</xml_diff>